<commit_message>
update the test result
</commit_message>
<xml_diff>
--- a/test_data_sheet.xlsx
+++ b/test_data_sheet.xlsx
@@ -480,7 +480,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Login Successful</t>
+          <t>Invalid Login. Try again.</t>
         </is>
       </c>
     </row>
@@ -529,12 +529,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Invalid Login. Try again.</t>
+          <t>Please fill in this field</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Exception: Frame.fill() missing 1 required positional argument: 'value'</t>
+          <t>Please fill in this field.</t>
         </is>
       </c>
     </row>
@@ -556,12 +556,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Invalid Login. Try again.</t>
+          <t>Please fill in this field</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Exception: Frame.fill() missing 1 required positional argument: 'value'</t>
+          <t>Please fill in this field.</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Exception: Locator.fill: value: expected string, got number</t>
+          <t>Invalid Login. Try again.</t>
         </is>
       </c>
     </row>
@@ -606,12 +606,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Invalid Login. Try again.</t>
+          <t>Please fill in this field</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Exception: Frame.fill() missing 1 required positional argument: 'value'</t>
+          <t>Please fill in this field.</t>
         </is>
       </c>
     </row>

</xml_diff>